<commit_message>
Custo da dívida pelo spread de crédito e prêmio de risco com risco-país
</commit_message>
<xml_diff>
--- a/4. Dados Gerdau/Database Valuation Gerdau.xlsx
+++ b/4. Dados Gerdau/Database Valuation Gerdau.xlsx
@@ -12,6 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Preços diários" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Macro anual" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expectativas Focus" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercado nas datas" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Retornos EUA (anual)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -74281,4 +74283,1867 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Data-base</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Spread Baa − Treasury 10 anos, mês anterior (%)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>EMBI+ Brasil, véspera (%)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Data do EMBI usado</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Receita no Brasil, último exercício (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>44252</v>
+      </c>
+      <c r="B2" s="7" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="C2" s="7" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>44251</v>
+      </c>
+      <c r="E2" s="7" t="n">
+        <v>42.9</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>44616</v>
+      </c>
+      <c r="B3" s="7" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="C3" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>44615</v>
+      </c>
+      <c r="E3" s="7" t="n">
+        <v>48.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>44987</v>
+      </c>
+      <c r="B4" s="7" t="n">
+        <v>1.84</v>
+      </c>
+      <c r="C4" s="7" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>44986</v>
+      </c>
+      <c r="E4" s="7" t="n">
+        <v>44.2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>45343</v>
+      </c>
+      <c r="B5" s="7" t="n">
+        <v>1.62</v>
+      </c>
+      <c r="C5" s="7" t="n">
+        <v>2.07</v>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>45342</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>40.2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>45708</v>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>45503</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>43.7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C155"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="36" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ano</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Ações EUA: índice de retorno total real em dez</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Títulos 10 anos EUA: índice de retorno total real em dez</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1871</v>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>132.2829539118026</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>1.031330727999685</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>1872</v>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>146.3260775899622</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>1.048389567421099</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>1873</v>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>144.8207943076529</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>1.18456517573235</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>1874</v>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>169.1106012612237</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>1.360000418499028</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>1875</v>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>183.7525697491768</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>1.559154760414039</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>1876</v>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>164.9953698435838</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>1.682633050919033</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>1877</v>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>182.7707783911895</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>2.004867780591919</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>1878</v>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>238.243028363378</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>2.456783428273355</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>1879</v>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>300.123123305479</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>2.192955207681907</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>1880</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>379.935316408855</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>2.385396859492788</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="n">
+        <v>1881</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>382.8949601754986</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>2.331804027808352</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>1882</v>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>400.2514789171279</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>2.46326636716714</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>1883</v>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>419.6984676671388</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>2.766666589524873</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>1884</v>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>406.8352695312659</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>3.221657548772257</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>1885</v>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>523.4135257821629</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>3.415196720048621</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>1886</v>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>621.4036739579029</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>3.667960157368911</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>1887</v>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>571.151981685087</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>3.538437195116861</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>1888</v>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>583.2239151406872</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>3.725540942824794</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>1889</v>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>668.0165138690729</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>4.106566537978267</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>1890</v>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>595.0270802729389</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>4.1383457464841</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="n">
+        <v>1891</v>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>768.1223098561372</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>4.508132747916636</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>1892</v>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>805.2931927231837</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>4.565724242397063</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>1893</v>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>733.9051315155197</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>5.137321195415279</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>1894</v>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>808.3713430894298</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>5.81905527974076</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="n">
+        <v>1895</v>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>824.8321053630897</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>5.804520814331399</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="n">
+        <v>1896</v>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>853.6724999144094</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>6.18615958619799</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="n">
+        <v>1897</v>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1000.66890543773</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>6.432304357982614</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="n">
+        <v>1898</v>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1218.687958864728</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>6.681622856660114</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="n">
+        <v>1899</v>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1147.615911896415</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>5.884041353198449</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="n">
+        <v>1900</v>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>1417.145588904676</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>6.320905039363542</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="n">
+        <v>1901</v>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>1624.993911076915</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>6.174745576020542</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n">
+        <v>1902</v>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>1596.23245097183</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>5.893340121843948</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n">
+        <v>1903</v>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>1446.925194711228</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>6.396540678701288</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n">
+        <v>1904</v>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>1818.69976464529</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>6.278861705184741</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n">
+        <v>1905</v>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2179.479336494765</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>6.520932422042152</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n">
+        <v>1906</v>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>2211.312350642731</v>
+      </c>
+      <c r="C37" s="5" t="n">
+        <v>6.281100474191055</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n">
+        <v>1907</v>
+      </c>
+      <c r="B38" s="5" t="n">
+        <v>1593.366175366124</v>
+      </c>
+      <c r="C38" s="5" t="n">
+        <v>6.551319392295588</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="n">
+        <v>1908</v>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>2239.211203478268</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>6.637288076964356</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="n">
+        <v>1909</v>
+      </c>
+      <c r="B40" s="5" t="n">
+        <v>2413.399300169656</v>
+      </c>
+      <c r="C40" s="5" t="n">
+        <v>6.173058412927729</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="n">
+        <v>1910</v>
+      </c>
+      <c r="B41" s="5" t="n">
+        <v>2410.275432514353</v>
+      </c>
+      <c r="C41" s="5" t="n">
+        <v>6.906602185745193</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="n">
+        <v>1911</v>
+      </c>
+      <c r="B42" s="5" t="n">
+        <v>2606.527494920548</v>
+      </c>
+      <c r="C42" s="5" t="n">
+        <v>7.318706423989944</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="n">
+        <v>1912</v>
+      </c>
+      <c r="B43" s="5" t="n">
+        <v>2627.207450087517</v>
+      </c>
+      <c r="C43" s="5" t="n">
+        <v>6.877708850292884</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="n">
+        <v>1913</v>
+      </c>
+      <c r="B44" s="5" t="n">
+        <v>2312.219400177417</v>
+      </c>
+      <c r="C44" s="5" t="n">
+        <v>7.099381855017745</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="n">
+        <v>1914</v>
+      </c>
+      <c r="B45" s="5" t="n">
+        <v>2213.862531679308</v>
+      </c>
+      <c r="C45" s="5" t="n">
+        <v>7.300492897837247</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="n">
+        <v>1915</v>
+      </c>
+      <c r="B46" s="5" t="n">
+        <v>2947.793752782796</v>
+      </c>
+      <c r="C46" s="5" t="n">
+        <v>7.564583149497632</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="n">
+        <v>1916</v>
+      </c>
+      <c r="B47" s="5" t="n">
+        <v>2852.21151807262</v>
+      </c>
+      <c r="C47" s="5" t="n">
+        <v>6.914834097353658</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="n">
+        <v>1917</v>
+      </c>
+      <c r="B48" s="5" t="n">
+        <v>1806.704151962622</v>
+      </c>
+      <c r="C48" s="5" t="n">
+        <v>5.957362848791683</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="n">
+        <v>1918</v>
+      </c>
+      <c r="B49" s="5" t="n">
+        <v>1893.316604363882</v>
+      </c>
+      <c r="C49" s="5" t="n">
+        <v>5.190517701378464</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="n">
+        <v>1919</v>
+      </c>
+      <c r="B50" s="5" t="n">
+        <v>1986.874306053089</v>
+      </c>
+      <c r="C50" s="5" t="n">
+        <v>4.59166029264108</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="n">
+        <v>1920</v>
+      </c>
+      <c r="B51" s="5" t="n">
+        <v>1577.286023437328</v>
+      </c>
+      <c r="C51" s="5" t="n">
+        <v>4.648550431759416</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="n">
+        <v>1921</v>
+      </c>
+      <c r="B52" s="5" t="n">
+        <v>2036.916696709612</v>
+      </c>
+      <c r="C52" s="5" t="n">
+        <v>5.783922310941281</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="n">
+        <v>1922</v>
+      </c>
+      <c r="B53" s="5" t="n">
+        <v>2653.889349909518</v>
+      </c>
+      <c r="C53" s="5" t="n">
+        <v>6.1875700270327</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="n">
+        <v>1923</v>
+      </c>
+      <c r="B54" s="5" t="n">
+        <v>2682.891426318554</v>
+      </c>
+      <c r="C54" s="5" t="n">
+        <v>6.444881843514208</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="n">
+        <v>1924</v>
+      </c>
+      <c r="B55" s="5" t="n">
+        <v>3384.46304582349</v>
+      </c>
+      <c r="C55" s="5" t="n">
+        <v>6.821380838581582</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="n">
+        <v>1925</v>
+      </c>
+      <c r="B56" s="5" t="n">
+        <v>4224.653466183729</v>
+      </c>
+      <c r="C56" s="5" t="n">
+        <v>6.950290090187822</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="n">
+        <v>1926</v>
+      </c>
+      <c r="B57" s="5" t="n">
+        <v>4870.057206405077</v>
+      </c>
+      <c r="C57" s="5" t="n">
+        <v>7.483371997554026</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="n">
+        <v>1927</v>
+      </c>
+      <c r="B58" s="5" t="n">
+        <v>6765.800618237719</v>
+      </c>
+      <c r="C58" s="5" t="n">
+        <v>7.940935459296649</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="n">
+        <v>1928</v>
+      </c>
+      <c r="B59" s="5" t="n">
+        <v>9454.873524701678</v>
+      </c>
+      <c r="C59" s="5" t="n">
+        <v>8.144197849014661</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="n">
+        <v>1929</v>
+      </c>
+      <c r="B60" s="5" t="n">
+        <v>9004.533408583706</v>
+      </c>
+      <c r="C60" s="5" t="n">
+        <v>8.568556106799271</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="n">
+        <v>1930</v>
+      </c>
+      <c r="B61" s="5" t="n">
+        <v>7309.767149292642</v>
+      </c>
+      <c r="C61" s="5" t="n">
+        <v>9.445817658604589</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="n">
+        <v>1931</v>
+      </c>
+      <c r="B62" s="5" t="n">
+        <v>4693.314150604848</v>
+      </c>
+      <c r="C62" s="5" t="n">
+        <v>10.5027727754883</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="n">
+        <v>1932</v>
+      </c>
+      <c r="B63" s="5" t="n">
+        <v>4652.965285874235</v>
+      </c>
+      <c r="C63" s="5" t="n">
+        <v>12.44456058391118</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="n">
+        <v>1933</v>
+      </c>
+      <c r="B64" s="5" t="n">
+        <v>7130.54538102877</v>
+      </c>
+      <c r="C64" s="5" t="n">
+        <v>12.97923694783029</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="n">
+        <v>1934</v>
+      </c>
+      <c r="B65" s="5" t="n">
+        <v>6827.436847306949</v>
+      </c>
+      <c r="C65" s="5" t="n">
+        <v>13.53735955729016</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="n">
+        <v>1935</v>
+      </c>
+      <c r="B66" s="5" t="n">
+        <v>9746.456625424518</v>
+      </c>
+      <c r="C66" s="5" t="n">
+        <v>13.69294117305178</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="n">
+        <v>1936</v>
+      </c>
+      <c r="B67" s="5" t="n">
+        <v>13041.85619647536</v>
+      </c>
+      <c r="C67" s="5" t="n">
+        <v>13.84205029837318</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="n">
+        <v>1937</v>
+      </c>
+      <c r="B68" s="5" t="n">
+        <v>8631.005289335368</v>
+      </c>
+      <c r="C68" s="5" t="n">
+        <v>13.94618476019214</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="n">
+        <v>1938</v>
+      </c>
+      <c r="B69" s="5" t="n">
+        <v>10873.66921344002</v>
+      </c>
+      <c r="C69" s="5" t="n">
+        <v>14.95643585921058</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="n">
+        <v>1939</v>
+      </c>
+      <c r="B70" s="5" t="n">
+        <v>11092.25946103782</v>
+      </c>
+      <c r="C70" s="5" t="n">
+        <v>15.51472400679824</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="n">
+        <v>1940</v>
+      </c>
+      <c r="B71" s="5" t="n">
+        <v>9949.139787612879</v>
+      </c>
+      <c r="C71" s="5" t="n">
+        <v>16.08942914430133</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="n">
+        <v>1941</v>
+      </c>
+      <c r="B72" s="5" t="n">
+        <v>8078.275385956423</v>
+      </c>
+      <c r="C72" s="5" t="n">
+        <v>14.3719501307301</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="n">
+        <v>1942</v>
+      </c>
+      <c r="B73" s="5" t="n">
+        <v>8680.446868429673</v>
+      </c>
+      <c r="C73" s="5" t="n">
+        <v>13.44816055870754</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="n">
+        <v>1943</v>
+      </c>
+      <c r="B74" s="5" t="n">
+        <v>10707.63061314361</v>
+      </c>
+      <c r="C74" s="5" t="n">
+        <v>13.37678845960763</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="n">
+        <v>1944</v>
+      </c>
+      <c r="B75" s="5" t="n">
+        <v>12562.3260060885</v>
+      </c>
+      <c r="C75" s="5" t="n">
+        <v>13.5167886002512</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="n">
+        <v>1945</v>
+      </c>
+      <c r="B76" s="5" t="n">
+        <v>16972.15894565032</v>
+      </c>
+      <c r="C76" s="5" t="n">
+        <v>13.73722864279812</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="n">
+        <v>1946</v>
+      </c>
+      <c r="B77" s="5" t="n">
+        <v>13061.72726931978</v>
+      </c>
+      <c r="C77" s="5" t="n">
+        <v>11.84669061466636</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="n">
+        <v>1947</v>
+      </c>
+      <c r="B78" s="5" t="n">
+        <v>12539.07696664722</v>
+      </c>
+      <c r="C78" s="5" t="n">
+        <v>10.96538261825942</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="n">
+        <v>1948</v>
+      </c>
+      <c r="B79" s="5" t="n">
+        <v>13011.44868193912</v>
+      </c>
+      <c r="C79" s="5" t="n">
+        <v>11.00375108445089</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="n">
+        <v>1949</v>
+      </c>
+      <c r="B80" s="5" t="n">
+        <v>15475.19415280353</v>
+      </c>
+      <c r="C80" s="5" t="n">
+        <v>11.50145192089544</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="n">
+        <v>1950</v>
+      </c>
+      <c r="B81" s="5" t="n">
+        <v>18680.31695008045</v>
+      </c>
+      <c r="C81" s="5" t="n">
+        <v>10.89997196063665</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="n">
+        <v>1951</v>
+      </c>
+      <c r="B82" s="5" t="n">
+        <v>22345.50374936518</v>
+      </c>
+      <c r="C82" s="5" t="n">
+        <v>10.44335813140258</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="n">
+        <v>1952</v>
+      </c>
+      <c r="B83" s="5" t="n">
+        <v>26152.78660427281</v>
+      </c>
+      <c r="C83" s="5" t="n">
+        <v>10.51798469321476</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="n">
+        <v>1953</v>
+      </c>
+      <c r="B84" s="5" t="n">
+        <v>26214.9863083162</v>
+      </c>
+      <c r="C84" s="5" t="n">
+        <v>10.95337254567381</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="n">
+        <v>1954</v>
+      </c>
+      <c r="B85" s="5" t="n">
+        <v>39103.48293913453</v>
+      </c>
+      <c r="C85" s="5" t="n">
+        <v>11.38236757854449</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="n">
+        <v>1955</v>
+      </c>
+      <c r="B86" s="5" t="n">
+        <v>52574.48506185009</v>
+      </c>
+      <c r="C86" s="5" t="n">
+        <v>11.21263902544188</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="3" t="n">
+        <v>1956</v>
+      </c>
+      <c r="B87" s="5" t="n">
+        <v>54272.93984192856</v>
+      </c>
+      <c r="C87" s="5" t="n">
+        <v>10.64877866830557</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="3" t="n">
+        <v>1957</v>
+      </c>
+      <c r="B88" s="5" t="n">
+        <v>47649.62659233629</v>
+      </c>
+      <c r="C88" s="5" t="n">
+        <v>11.07621037618423</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="3" t="n">
+        <v>1958</v>
+      </c>
+      <c r="B89" s="5" t="n">
+        <v>64515.49722758618</v>
+      </c>
+      <c r="C89" s="5" t="n">
+        <v>10.6476147583773</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="3" t="n">
+        <v>1959</v>
+      </c>
+      <c r="B90" s="5" t="n">
+        <v>72243.19996026858</v>
+      </c>
+      <c r="C90" s="5" t="n">
+        <v>10.21351999494286</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="n">
+        <v>1960</v>
+      </c>
+      <c r="B91" s="5" t="n">
+        <v>70963.52993866903</v>
+      </c>
+      <c r="C91" s="5" t="n">
+        <v>11.2464663126154</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="3" t="n">
+        <v>1961</v>
+      </c>
+      <c r="B92" s="5" t="n">
+        <v>91704.55444351272</v>
+      </c>
+      <c r="C92" s="5" t="n">
+        <v>11.40281374106578</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="n">
+        <v>1962</v>
+      </c>
+      <c r="B93" s="5" t="n">
+        <v>81700.69070857765</v>
+      </c>
+      <c r="C93" s="5" t="n">
+        <v>11.8988294185275</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="3" t="n">
+        <v>1963</v>
+      </c>
+      <c r="B94" s="5" t="n">
+        <v>98214.07258635695</v>
+      </c>
+      <c r="C94" s="5" t="n">
+        <v>11.9152592555613</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="n">
+        <v>1964</v>
+      </c>
+      <c r="B95" s="5" t="n">
+        <v>113393.6344368136</v>
+      </c>
+      <c r="C95" s="5" t="n">
+        <v>12.25396052444982</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="n">
+        <v>1965</v>
+      </c>
+      <c r="B96" s="5" t="n">
+        <v>125207.9992279365</v>
+      </c>
+      <c r="C96" s="5" t="n">
+        <v>12.10888032499875</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="n">
+        <v>1966</v>
+      </c>
+      <c r="B97" s="5" t="n">
+        <v>110935.9467590718</v>
+      </c>
+      <c r="C97" s="5" t="n">
+        <v>12.07541237413273</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="3" t="n">
+        <v>1967</v>
+      </c>
+      <c r="B98" s="5" t="n">
+        <v>130207.8097364532</v>
+      </c>
+      <c r="C98" s="5" t="n">
+        <v>11.52717669772548</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="n">
+        <v>1968</v>
+      </c>
+      <c r="B99" s="5" t="n">
+        <v>143240.6685084044</v>
+      </c>
+      <c r="C99" s="5" t="n">
+        <v>11.35428702193641</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="3" t="n">
+        <v>1969</v>
+      </c>
+      <c r="B100" s="5" t="n">
+        <v>119140.4057509456</v>
+      </c>
+      <c r="C100" s="5" t="n">
+        <v>10.15746881544798</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="n">
+        <v>1970</v>
+      </c>
+      <c r="B101" s="5" t="n">
+        <v>115886.7531411201</v>
+      </c>
+      <c r="C101" s="5" t="n">
+        <v>11.31770226852989</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="3" t="n">
+        <v>1971</v>
+      </c>
+      <c r="B102" s="5" t="n">
+        <v>127542.8540597427</v>
+      </c>
+      <c r="C102" s="5" t="n">
+        <v>12.04881413694796</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="n">
+        <v>1972</v>
+      </c>
+      <c r="B103" s="5" t="n">
+        <v>150326.2479848707</v>
+      </c>
+      <c r="C103" s="5" t="n">
+        <v>12.00249113732713</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="3" t="n">
+        <v>1973</v>
+      </c>
+      <c r="B104" s="5" t="n">
+        <v>114974.1097051091</v>
+      </c>
+      <c r="C104" s="5" t="n">
+        <v>11.49199694583022</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="n">
+        <v>1974</v>
+      </c>
+      <c r="B105" s="5" t="n">
+        <v>75639.02025997124</v>
+      </c>
+      <c r="C105" s="5" t="n">
+        <v>10.49464914706582</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="3" t="n">
+        <v>1975</v>
+      </c>
+      <c r="B106" s="5" t="n">
+        <v>97641.40645219802</v>
+      </c>
+      <c r="C106" s="5" t="n">
+        <v>10.20785215975327</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="3" t="n">
+        <v>1976</v>
+      </c>
+      <c r="B107" s="5" t="n">
+        <v>114079.6615851373</v>
+      </c>
+      <c r="C107" s="5" t="n">
+        <v>11.36636267821457</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="n">
+        <v>1977</v>
+      </c>
+      <c r="B108" s="5" t="n">
+        <v>100173.9712943629</v>
+      </c>
+      <c r="C108" s="5" t="n">
+        <v>10.81981184096514</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="n">
+        <v>1978</v>
+      </c>
+      <c r="B109" s="5" t="n">
+        <v>99074.27812793432</v>
+      </c>
+      <c r="C109" s="5" t="n">
+        <v>9.867497383364595</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="3" t="n">
+        <v>1979</v>
+      </c>
+      <c r="B110" s="5" t="n">
+        <v>103329.5629062424</v>
+      </c>
+      <c r="C110" s="5" t="n">
+        <v>8.752967516406605</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="3" t="n">
+        <v>1980</v>
+      </c>
+      <c r="B111" s="5" t="n">
+        <v>119596.0143314959</v>
+      </c>
+      <c r="C111" s="5" t="n">
+        <v>7.509726371092225</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="n">
+        <v>1981</v>
+      </c>
+      <c r="B112" s="5" t="n">
+        <v>107055.1892056114</v>
+      </c>
+      <c r="C112" s="5" t="n">
+        <v>7.524460698345904</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="n">
+        <v>1982</v>
+      </c>
+      <c r="B113" s="5" t="n">
+        <v>122907.6013676822</v>
+      </c>
+      <c r="C113" s="5" t="n">
+        <v>9.88855765435706</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="3" t="n">
+        <v>1983</v>
+      </c>
+      <c r="B114" s="5" t="n">
+        <v>145856.7027093157</v>
+      </c>
+      <c r="C114" s="5" t="n">
+        <v>9.842306240921772</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="3" t="n">
+        <v>1984</v>
+      </c>
+      <c r="B115" s="5" t="n">
+        <v>146941.608926751</v>
+      </c>
+      <c r="C115" s="5" t="n">
+        <v>10.91547749582364</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="n">
+        <v>1985</v>
+      </c>
+      <c r="B116" s="5" t="n">
+        <v>185955.2952990697</v>
+      </c>
+      <c r="C116" s="5" t="n">
+        <v>13.41993486152435</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="n">
+        <v>1986</v>
+      </c>
+      <c r="B117" s="5" t="n">
+        <v>228299.7978512901</v>
+      </c>
+      <c r="C117" s="5" t="n">
+        <v>16.56595536963849</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="n">
+        <v>1987</v>
+      </c>
+      <c r="B118" s="5" t="n">
+        <v>218376.3208372329</v>
+      </c>
+      <c r="C118" s="5" t="n">
+        <v>15.13420638766222</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="n">
+        <v>1988</v>
+      </c>
+      <c r="B119" s="5" t="n">
+        <v>248442.2837514736</v>
+      </c>
+      <c r="C119" s="5" t="n">
+        <v>15.69442454913491</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="n">
+        <v>1989</v>
+      </c>
+      <c r="B120" s="5" t="n">
+        <v>309132.3734866644</v>
+      </c>
+      <c r="C120" s="5" t="n">
+        <v>17.77008676239673</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="n">
+        <v>1990</v>
+      </c>
+      <c r="B121" s="5" t="n">
+        <v>284495.6300837969</v>
+      </c>
+      <c r="C121" s="5" t="n">
+        <v>17.92830100274471</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="n">
+        <v>1991</v>
+      </c>
+      <c r="B122" s="5" t="n">
+        <v>336956.9557697553</v>
+      </c>
+      <c r="C122" s="5" t="n">
+        <v>20.15245772336195</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="n">
+        <v>1992</v>
+      </c>
+      <c r="B123" s="5" t="n">
+        <v>378232.9369536712</v>
+      </c>
+      <c r="C123" s="5" t="n">
+        <v>21.47998605453914</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="n">
+        <v>1993</v>
+      </c>
+      <c r="B124" s="5" t="n">
+        <v>404781.3482461053</v>
+      </c>
+      <c r="C124" s="5" t="n">
+        <v>23.85888954016531</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="n">
+        <v>1994</v>
+      </c>
+      <c r="B125" s="5" t="n">
+        <v>396036.8883407941</v>
+      </c>
+      <c r="C125" s="5" t="n">
+        <v>21.49083251595152</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="n">
+        <v>1995</v>
+      </c>
+      <c r="B126" s="5" t="n">
+        <v>534622.4481516506</v>
+      </c>
+      <c r="C126" s="5" t="n">
+        <v>26.04354885992753</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="n">
+        <v>1996</v>
+      </c>
+      <c r="B127" s="5" t="n">
+        <v>639352.7682516751</v>
+      </c>
+      <c r="C127" s="5" t="n">
+        <v>25.69483562153838</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="n">
+        <v>1997</v>
+      </c>
+      <c r="B128" s="5" t="n">
+        <v>828382.3866024488</v>
+      </c>
+      <c r="C128" s="5" t="n">
+        <v>27.91005541524141</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="3" t="n">
+        <v>1998</v>
+      </c>
+      <c r="B129" s="5" t="n">
+        <v>1023066.58814785</v>
+      </c>
+      <c r="C129" s="5" t="n">
+        <v>31.65707079572593</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="3" t="n">
+        <v>1999</v>
+      </c>
+      <c r="B130" s="5" t="n">
+        <v>1211106.233200189</v>
+      </c>
+      <c r="C130" s="5" t="n">
+        <v>28.75044801958864</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="3" t="n">
+        <v>2000</v>
+      </c>
+      <c r="B131" s="5" t="n">
+        <v>1104021.645416953</v>
+      </c>
+      <c r="C131" s="5" t="n">
+        <v>31.92557241531178</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="n">
+        <v>2001</v>
+      </c>
+      <c r="B132" s="5" t="n">
+        <v>947771.7243653137</v>
+      </c>
+      <c r="C132" s="5" t="n">
+        <v>33.41716404394907</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="3" t="n">
+        <v>2002</v>
+      </c>
+      <c r="B133" s="5" t="n">
+        <v>738890.9827939284</v>
+      </c>
+      <c r="C133" s="5" t="n">
+        <v>37.18030387689463</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="3" t="n">
+        <v>2003</v>
+      </c>
+      <c r="B134" s="5" t="n">
+        <v>886724.6334423319</v>
+      </c>
+      <c r="C134" s="5" t="n">
+        <v>37.19631381076803</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="3" t="n">
+        <v>2004</v>
+      </c>
+      <c r="B135" s="5" t="n">
+        <v>968826.8158190306</v>
+      </c>
+      <c r="C135" s="5" t="n">
+        <v>37.6829055919445</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="3" t="n">
+        <v>2005</v>
+      </c>
+      <c r="B136" s="5" t="n">
+        <v>1003207.019770566</v>
+      </c>
+      <c r="C136" s="5" t="n">
+        <v>37.28394375735243</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="3" t="n">
+        <v>2006</v>
+      </c>
+      <c r="B137" s="5" t="n">
+        <v>1117927.32175778</v>
+      </c>
+      <c r="C137" s="5" t="n">
+        <v>37.85526118584974</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="3" t="n">
+        <v>2007</v>
+      </c>
+      <c r="B138" s="5" t="n">
+        <v>1141903.296300477</v>
+      </c>
+      <c r="C138" s="5" t="n">
+        <v>39.51144670079425</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="3" t="n">
+        <v>2008</v>
+      </c>
+      <c r="B139" s="5" t="n">
+        <v>693268.8429337239</v>
+      </c>
+      <c r="C139" s="5" t="n">
+        <v>47.12885167016712</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="3" t="n">
+        <v>2009</v>
+      </c>
+      <c r="B140" s="5" t="n">
+        <v>877576.2400976805</v>
+      </c>
+      <c r="C140" s="5" t="n">
+        <v>42.80583190974063</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="3" t="n">
+        <v>2010</v>
+      </c>
+      <c r="B141" s="5" t="n">
+        <v>985833.1485441992</v>
+      </c>
+      <c r="C141" s="5" t="n">
+        <v>44.61473230182818</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="3" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B142" s="5" t="n">
+        <v>977619.0875342324</v>
+      </c>
+      <c r="C142" s="5" t="n">
+        <v>49.91682863827565</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B143" s="5" t="n">
+        <v>1122310.401693501</v>
+      </c>
+      <c r="C143" s="5" t="n">
+        <v>51.13395630418523</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="3" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B144" s="5" t="n">
+        <v>1434263.884588291</v>
+      </c>
+      <c r="C144" s="5" t="n">
+        <v>46.38297800129055</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="3" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B145" s="5" t="n">
+        <v>1649309.984365149</v>
+      </c>
+      <c r="C145" s="5" t="n">
+        <v>50.16693560359909</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B146" s="5" t="n">
+        <v>1670733.322276079</v>
+      </c>
+      <c r="C146" s="5" t="n">
+        <v>50.71314850382903</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B147" s="5" t="n">
+        <v>1828793.867397628</v>
+      </c>
+      <c r="C147" s="5" t="n">
+        <v>49.4468253305144</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B148" s="5" t="n">
+        <v>2165559.717981845</v>
+      </c>
+      <c r="C148" s="5" t="n">
+        <v>49.9529949096847</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B149" s="5" t="n">
+        <v>2086274.605957681</v>
+      </c>
+      <c r="C149" s="5" t="n">
+        <v>48.56964450775431</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B150" s="5" t="n">
+        <v>2573097.405342015</v>
+      </c>
+      <c r="C150" s="5" t="n">
+        <v>52.83562267600085</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="n">
+        <v>2020</v>
+      </c>
+      <c r="B151" s="5" t="n">
+        <v>3008117.088570186</v>
+      </c>
+      <c r="C151" s="5" t="n">
+        <v>57.29450706953979</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="3" t="n">
+        <v>2021</v>
+      </c>
+      <c r="B152" s="5" t="n">
+        <v>3604596.800959033</v>
+      </c>
+      <c r="C152" s="5" t="n">
+        <v>51.58103737192001</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="3" t="n">
+        <v>2022</v>
+      </c>
+      <c r="B153" s="5" t="n">
+        <v>2878645.255049742</v>
+      </c>
+      <c r="C153" s="5" t="n">
+        <v>41.18234160812391</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="3" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B154" s="5" t="n">
+        <v>3389468.321562686</v>
+      </c>
+      <c r="C154" s="5" t="n">
+        <v>40.05416842439841</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="3" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B155" s="5" t="n">
+        <v>4283497.296167756</v>
+      </c>
+      <c r="C155" s="5" t="n">
+        <v>39.3626792932078</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Taxa livre de risco pela NTN-F menos o EMBI
</commit_message>
<xml_diff>
--- a/4. Dados Gerdau/Database Valuation Gerdau.xlsx
+++ b/4. Dados Gerdau/Database Valuation Gerdau.xlsx
@@ -74291,7 +74291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -74299,6 +74299,8 @@
     <col width="15" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -74309,20 +74311,30 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>NTN-F mais longa, véspera (% a.a.)</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Vencimento da NTN-F usada</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Spread Baa − Treasury 10 anos, mês anterior (%)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EMBI+ Brasil, véspera (%)</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Data do EMBI usado</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Receita no Brasil, último exercício (%)</t>
         </is>
@@ -74333,15 +74345,21 @@
         <v>44252</v>
       </c>
       <c r="B2" s="7" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>47849</v>
+      </c>
+      <c r="D2" s="7" t="n">
         <v>2.16</v>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="E2" s="7" t="n">
         <v>2.8</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="F2" s="2" t="n">
         <v>44251</v>
       </c>
-      <c r="E2" s="7" t="n">
+      <c r="G2" s="7" t="n">
         <v>42.9</v>
       </c>
     </row>
@@ -74350,15 +74368,21 @@
         <v>44616</v>
       </c>
       <c r="B3" s="7" t="n">
+        <v>11.58</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>48580</v>
+      </c>
+      <c r="D3" s="7" t="n">
         <v>1.82</v>
       </c>
-      <c r="C3" s="7" t="n">
+      <c r="E3" s="7" t="n">
         <v>3.4</v>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="F3" s="2" t="n">
         <v>44615</v>
       </c>
-      <c r="E3" s="7" t="n">
+      <c r="G3" s="7" t="n">
         <v>48.2</v>
       </c>
     </row>
@@ -74367,15 +74391,21 @@
         <v>44987</v>
       </c>
       <c r="B4" s="7" t="n">
+        <v>13.35</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>48580</v>
+      </c>
+      <c r="D4" s="7" t="n">
         <v>1.84</v>
       </c>
-      <c r="C4" s="7" t="n">
+      <c r="E4" s="7" t="n">
         <v>2.47</v>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="F4" s="2" t="n">
         <v>44986</v>
       </c>
-      <c r="E4" s="7" t="n">
+      <c r="G4" s="7" t="n">
         <v>44.2</v>
       </c>
     </row>
@@ -74384,15 +74414,21 @@
         <v>45343</v>
       </c>
       <c r="B5" s="7" t="n">
+        <v>10.79</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>49310</v>
+      </c>
+      <c r="D5" s="7" t="n">
         <v>1.62</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="E5" s="7" t="n">
         <v>2.07</v>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="F5" s="2" t="n">
         <v>45342</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="G5" s="7" t="n">
         <v>40.2</v>
       </c>
     </row>
@@ -74401,15 +74437,21 @@
         <v>45708</v>
       </c>
       <c r="B6" s="7" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>49310</v>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>1.45</v>
       </c>
-      <c r="C6" s="7" t="n">
+      <c r="E6" s="7" t="n">
         <v>2.28</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="F6" s="2" t="n">
         <v>45503</v>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="G6" s="7" t="n">
         <v>43.7</v>
       </c>
     </row>

</xml_diff>